<commit_message>
Venue access & logistics fields (community features §2) (mirror of Hugo)
venues schema gains wheelchair/transit/parking/access; venue [slug] renders
the Getting there & access section; event [slug] shows the wheelchair badge
+ access link. STRINGS keys, both src and package copies. Shared importer +
sample workbook synced.
</commit_message>
<xml_diff>
--- a/scripts/sample-community.xlsx
+++ b/scripts/sample-community.xlsx
@@ -170,10 +170,30 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Wheelchair</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Transit</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Access</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -202,10 +222,30 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Two blocks from Central station.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Free street parking after 6pm.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Gender-neutral washrooms on level 2; quiet room on request.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>https://example.com</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
Community features §2: venue access fields (mirror of Hugo) (#39)
* Venue access & logistics fields (community features §2) (mirror of Hugo)

venues schema gains wheelchair/transit/parking/access; venue [slug] renders
the Getting there & access section; event [slug] shows the wheelchair badge
+ access link. STRINGS keys, both src and package copies. Shared importer +
sample workbook synced.

* Package venue single: import config from popular:config
</commit_message>
<xml_diff>
--- a/scripts/sample-community.xlsx
+++ b/scripts/sample-community.xlsx
@@ -170,10 +170,30 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Wheelchair</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Transit</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Access</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -202,10 +222,30 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Two blocks from Central station.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Free street parking after 6pm.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Gender-neutral washrooms on level 2; quiet room on request.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>https://example.com</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>